<commit_message>
Am rezolvat cerinta cu Architectural Design Phase Defects
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\anul3sem2\VVSS\lab\Lab01\CheckLists\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\otili\Desktop\AN_3\Sem2\VVSS\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D27F635-5056-4620-9869-4387D55B96B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="11496" tabRatio="650"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="650" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -17,25 +18,12 @@
     <sheet name="Coding Phase Defects" sheetId="5" r:id="rId3"/>
     <sheet name="Tool-basedCodeAnalysis" sheetId="8" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -200,19 +188,95 @@
   </si>
   <si>
     <t>Se creează confuzie la procesarea comenzii. Nu e clar dacă funcționalitatea e pentru managementul stocului sau pentru calculul prețului unei băuturi pe baza ingredientelor.</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>A02</t>
+  </si>
+  <si>
+    <t>A03</t>
+  </si>
+  <si>
+    <t>A04</t>
+  </si>
+  <si>
+    <t>A05</t>
+  </si>
+  <si>
+    <t>A06</t>
+  </si>
+  <si>
+    <t>A07</t>
+  </si>
+  <si>
+    <t>A08</t>
+  </si>
+  <si>
+    <t>A09</t>
+  </si>
+  <si>
+    <t>Structura pe straturi Controller-Service-Repo e vizibila</t>
+  </si>
+  <si>
+    <t>Separarea responsabilitatilor intre layere este clar evidentiata</t>
+  </si>
+  <si>
+    <t>Autentificarea și gestionarea utilizatorilor/rolurilor (Admin/Chelner)</t>
+  </si>
+  <si>
+    <t>Lipseste logica de persistenta a rapoartelor zilnice</t>
+  </si>
+  <si>
+    <t>DrinkShopService nu permite o comanda cu mai multe bauturi (produse).</t>
+  </si>
+  <si>
+    <t>Nemeș Otilia, Pașca Valentina - Diana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intre ValidationException si DrinkShopService nu exista nici o relatie. </t>
+  </si>
+  <si>
+    <t>Se utilizează Repository Pattern pentru persistență și Validator Pattern pentru regulile de business.</t>
+  </si>
+  <si>
+    <t>Denumirile sunt sugestive (ex: FileRetetaRepository)</t>
+  </si>
+  <si>
+    <t>DrinkShopController preia prea multe sarcini ce ar putea fi redistribuite.</t>
+  </si>
+  <si>
+    <t>Intre DrinkShopApp si DrinkShopController lipseste asocierea.</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>Lipseste enum-ul pentru unitatea de masura a ingredientelor.</t>
+  </si>
+  <si>
+    <t>Pașca Valentina - Diana</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="12" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -398,83 +462,85 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="20" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,9 +559,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -533,9 +599,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -570,7 +636,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -605,7 +671,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -778,7 +844,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
@@ -800,19 +866,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -825,7 +891,7 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>35</v>
       </c>
       <c r="J3" s="17">
@@ -836,14 +902,14 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="27"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>36</v>
       </c>
       <c r="J4" s="3">
@@ -854,10 +920,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="27"/>
+      <c r="E5" s="29"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -869,19 +935,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="22"/>
+      <c r="E6" s="24"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="22"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -901,10 +967,10 @@
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="23">
         <v>4</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -916,10 +982,10 @@
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="37" t="s">
+      <c r="D11" s="23" t="s">
         <v>46</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -931,10 +997,10 @@
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="37" t="s">
+      <c r="D12" s="23" t="s">
         <v>46</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -946,10 +1012,10 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="37" t="s">
+      <c r="C13" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="23" t="s">
         <v>49</v>
       </c>
       <c r="E13" s="2" t="s">
@@ -961,10 +1027,10 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="37">
+      <c r="D14" s="23">
         <v>7</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -976,10 +1042,10 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="37" t="s">
+      <c r="C15" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="37" t="s">
+      <c r="D15" s="23" t="s">
         <v>50</v>
       </c>
       <c r="E15" s="2" t="s">
@@ -991,10 +1057,10 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="23" t="s">
         <v>49</v>
       </c>
       <c r="E16" s="2" t="s">
@@ -1106,7 +1172,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1127,19 +1193,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1152,31 +1218,39 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
+      <c r="I3" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="17">
+        <v>235</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="28"/>
+      <c r="E4" s="30"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="J4" s="3">
+        <v>235</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="30"/>
+      <c r="E5" s="32"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1188,15 +1262,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="24"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
+      <c r="D7" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="24"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1212,103 +1290,147 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E10" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E11" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E12" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E13" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E14" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
+      <c r="C15" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="D15" s="1"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E15" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
+      <c r="C16" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E16" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
+      <c r="C17" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E17" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
+      <c r="C18" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="D18" s="1"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E18" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
+      <c r="C19" s="1" t="s">
+        <v>63</v>
+      </c>
       <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E19" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="1"/>
+      <c r="C20" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="D20" s="1"/>
-      <c r="E20" s="2"/>
+      <c r="E20" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
@@ -1369,7 +1491,9 @@
         <v>8</v>
       </c>
       <c r="D28" s="12"/>
-      <c r="E28" s="1"/>
+      <c r="E28" s="38">
+        <v>5.2083333333333336E-2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1386,7 +1510,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1408,19 +1532,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1440,10 +1564,10 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="31"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1454,10 +1578,10 @@
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="33"/>
+      <c r="E5" s="35"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1469,15 +1593,15 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1703,7 +1827,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
@@ -1726,19 +1850,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1758,8 +1882,8 @@
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1770,8 +1894,8 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1783,8 +1907,8 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -2014,11 +2138,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
       <c r="F32" s="18"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Am realizat partea de Coding Phase Defects.
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\otili\Desktop\AN_3\Sem2\VVSS\MyDrinkShop\docs\Lab01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D27F635-5056-4620-9869-4387D55B96B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="650" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="650" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -18,12 +17,12 @@
     <sheet name="Coding Phase Defects" sheetId="5" r:id="rId3"/>
     <sheet name="Tool-basedCodeAnalysis" sheetId="8" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="109">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -257,12 +256,105 @@
   </si>
   <si>
     <t>Pașca Valentina - Diana</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>C02</t>
+  </si>
+  <si>
+    <t>C03</t>
+  </si>
+  <si>
+    <t>C04</t>
+  </si>
+  <si>
+    <t>C05</t>
+  </si>
+  <si>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>C07</t>
+  </si>
+  <si>
+    <t>C08</t>
+  </si>
+  <si>
+    <t>C09</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>În constructorul clasei DrinkShopService, parametru din constructor numit stocService este de fapt un Repository și ar trebui redenumit stocRepo.</t>
+  </si>
+  <si>
+    <t>DrinkShopService, linia 23</t>
+  </si>
+  <si>
+    <t>DrinkShopService, linia 84</t>
+  </si>
+  <si>
+    <t>În clasa StocService, metoda consuma(Reteta reteta) efectuează un cast forțat la (int) atunci când actualizează cantitatea în obiectul Stoc, ceea ce duce la un management imprecis al stocului (ex: 1.5 kg - 0.7 kg va rezulta în 0 kg în loc de 0.8 kg).</t>
+  </si>
+  <si>
+    <t>StocService, 73</t>
+  </si>
+  <si>
+    <t>În DrinkShopService.comandaProdus, nu există o verificare dacă obiectul reteta returnat este null înainte de a fi utilizat.</t>
+  </si>
+  <si>
+    <t>În StocService, metoda consuma nu verifică dacă variabila ramas este 0 la finalul buclei. Dacă stocul se termină neașteptat, programul nu raportează eroarea corect.</t>
+  </si>
+  <si>
+    <t>StocService, 77</t>
+  </si>
+  <si>
+    <t>DrinkShopService, linia 86</t>
+  </si>
+  <si>
+    <t>FileOrderRepository, 31</t>
+  </si>
+  <si>
+    <t>RetetaValidator, 26</t>
+  </si>
+  <si>
+    <t>În clasa RetetaValidator.java, metoda validate folosește accumulateAndGet pentru a uni mesajele, fără a folosi un delimitator, în cazul în care sunt erori multiple.</t>
+  </si>
+  <si>
+    <t>Nu există riscuri de bucle infinite.</t>
+  </si>
+  <si>
+    <t>Apelurile metodelor între straturile aplicației Controller -&gt; Service -&gt; Repository respectă semnăturile definite în interfețe</t>
+  </si>
+  <si>
+    <t>Procesarea datelor de ieșire pentru generarea bonului fiscal și a rapoartelor zilnice funcționează conform cerințelor.</t>
+  </si>
+  <si>
+    <t>Nu e necesară în program indexarea manuală, deoarece se folosesc iterații moderne ca și streams.</t>
+  </si>
+  <si>
+    <t>Variabilele și constantele din proiect respectă convențiile de numire standard.</t>
+  </si>
+  <si>
+    <t>Am creat asociere 1 la 1 între Product și Reteta. Am actualizată diagrama, astfel încât să reflecte relația, asigurând o mapare corectă.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">În clasa FileOrderRepository.java, metoda extractEntity trebuie protejată cu un bloc try-catch. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -497,6 +589,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="20" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -539,8 +633,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -559,9 +651,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -599,9 +691,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -636,7 +728,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -671,7 +763,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -844,7 +936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
@@ -866,19 +958,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -902,10 +994,10 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="27"/>
+      <c r="E4" s="29"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -920,10 +1012,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="29"/>
+      <c r="E5" s="31"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -935,19 +1027,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="24"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="24"/>
+      <c r="E7" s="26"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1172,7 +1264,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1193,19 +1285,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1218,7 +1310,7 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="39" t="s">
+      <c r="I3" s="25" t="s">
         <v>36</v>
       </c>
       <c r="J3" s="17">
@@ -1229,14 +1321,14 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="30"/>
+      <c r="E4" s="32"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="39" t="s">
+      <c r="I4" s="25" t="s">
         <v>77</v>
       </c>
       <c r="J4" s="3">
@@ -1247,10 +1339,10 @@
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="32"/>
+      <c r="E5" s="34"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1262,19 +1354,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="E6" s="24"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="24"/>
+      <c r="E7" s="26"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1491,7 +1583,7 @@
         <v>8</v>
       </c>
       <c r="D28" s="12"/>
-      <c r="E28" s="38">
+      <c r="E28" s="24">
         <v>5.2083333333333336E-2</v>
       </c>
     </row>
@@ -1510,7 +1602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1532,19 +1624,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1557,31 +1649,39 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
+      <c r="I3" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="17">
+        <v>235</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="D4" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="33"/>
+      <c r="E4" s="35"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="3">
+        <v>235</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="35"/>
+      <c r="E5" s="37"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1593,15 +1693,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
+      <c r="D6" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
+      <c r="D7" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="26"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1617,112 +1721,184 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
+      <c r="C11" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C16" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C17" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C18" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C19" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C20" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="2"/>
+      <c r="C21" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="3">
@@ -1810,7 +1986,9 @@
         <v>8</v>
       </c>
       <c r="D32" s="12"/>
-      <c r="E32" s="1"/>
+      <c r="E32" s="24">
+        <v>6.25E-2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1827,7 +2005,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
@@ -1850,19 +2028,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1882,8 +2060,8 @@
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1894,8 +2072,8 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1907,8 +2085,8 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -2138,11 +2316,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="36" t="s">
+      <c r="C32" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="37"/>
-      <c r="E32" s="37"/>
+      <c r="D32" s="39"/>
+      <c r="E32" s="39"/>
       <c r="F32" s="18"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Am realizat evaluarea statica a calitatii codului
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\MyDrinkShop\docs\Lab01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\otili\Desktop\AN_3\Sem2\VVSS\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB9A22A8-E5F5-48D1-9F9F-D9B1B7C78AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="650" activeTab="2"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="650" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -17,12 +18,12 @@
     <sheet name="Coding Phase Defects" sheetId="5" r:id="rId3"/>
     <sheet name="Tool-basedCodeAnalysis" sheetId="8" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="144">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -120,9 +121,6 @@
     <t>Tool-based Code Analysis</t>
   </si>
   <si>
-    <t>Effort to perform tool-based code analysis (hours):</t>
-  </si>
-  <si>
     <t>03.04.2026</t>
   </si>
   <si>
@@ -349,19 +347,153 @@
   </si>
   <si>
     <t xml:space="preserve">În clasa FileOrderRepository.java, metoda extractEntity trebuie protejată cu un bloc try-catch. </t>
+  </si>
+  <si>
+    <t>Nemeș Otilia, Pașca Valentina Diana</t>
+  </si>
+  <si>
+    <t>05.03.2026</t>
+  </si>
+  <si>
+    <t>SonarQube</t>
+  </si>
+  <si>
+    <t>Pașca Valentina Diana</t>
+  </si>
+  <si>
+    <t>DailyReportService,23</t>
+  </si>
+  <si>
+    <t>This block of commented-out lines of code should be removed.</t>
+  </si>
+  <si>
+    <t>//        List&lt;Order&gt; orders = StreamSupport.stream(repo.findAll().spliterator(), false)
+//                .collect(Collectors.toList());</t>
+  </si>
+  <si>
+    <t>Codul a fost sters conform recomandarii.</t>
+  </si>
+  <si>
+    <t>DailyReportService, 6</t>
+  </si>
+  <si>
+    <t>DailyReportService, 7</t>
+  </si>
+  <si>
+    <t>DailyReportService, 8</t>
+  </si>
+  <si>
+    <t>Remove this unused import 'java.util.stream.Collectors'.</t>
+  </si>
+  <si>
+    <t>Remove this unused import 'java.util.stream.StreamSupport'.</t>
+  </si>
+  <si>
+    <t>import java.util.List;</t>
+  </si>
+  <si>
+    <t>import java.util.stream.Collectors;</t>
+  </si>
+  <si>
+    <t>import java.util.stream.StreamSupport;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this unused import </t>
+  </si>
+  <si>
+    <t>Order, 62</t>
+  </si>
+  <si>
+    <t>Update this method so that its implementation is not identical to "getTotalPrice" on line 33.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public double getTotal() {
+        return totalPrice;
+    } public double getTotalPrice() {
+        return totalPrice;
+    }
+</t>
+  </si>
+  <si>
+    <t>Am pastrat doar functia getTotalPrice() si am modificat peste tot in cod unde se folosea functia getTotal()</t>
+  </si>
+  <si>
+    <t>Repository, 5</t>
+  </si>
+  <si>
+    <t>Rename this generic name to match the regular expression '^[A-Z][0-9]?$'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public interface Repository&lt;ID, E&gt; </t>
+  </si>
+  <si>
+    <t>Nu am modificat: În acest context, utilizarea ID îmbunătățește lizibilitatea codului și clarifică rolul parametrului generic fără a induce confuzie.</t>
+  </si>
+  <si>
+    <t>AbstractRepository, 37</t>
+  </si>
+  <si>
+    <t>Update this method so that its implementation is not identical to "save" on line 26.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+    public E update(E entity) {
+        entities.put(getId(entity), entity);
+        return entity;
+    }
+       </t>
+  </si>
+  <si>
+    <t>public E update(E entity) {
+        if(entities.get(getId(entity)) == null) {
+            return null;
+        }
+        entities.put(getId(entity), entity);
+        return entity;
+    }</t>
+  </si>
+  <si>
+    <t>AbstractRepository, 21</t>
+  </si>
+  <si>
+    <t>//                    .collect(Collectors.toList());
+        // return (List&lt;E&gt;) entities.values();</t>
+  </si>
+  <si>
+    <t>Remove this unnecessary cast to "List".</t>
+  </si>
+  <si>
+    <t>AbstractRepository, 20</t>
+  </si>
+  <si>
+    <t>return (List&lt;E&gt;)StreamSupport.stream(entities.values().spliterator(), false).toList();</t>
+  </si>
+  <si>
+    <t xml:space="preserve">return StreamSupport.stream(entities.values().spliterator(), false).toList();
+   </t>
+  </si>
+  <si>
+    <t>Effort to perform tool-based code analysis (hours):  30 min</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="13" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -554,85 +686,86 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -651,9 +784,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -691,9 +824,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -728,7 +861,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -763,7 +896,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -936,7 +1069,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
@@ -965,12 +1098,12 @@
       <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -984,7 +1117,7 @@
         <v>20</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J3" s="17">
         <v>235</v>
@@ -994,15 +1127,15 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="32"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J4" s="3">
         <v>235</v>
@@ -1012,10 +1145,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="34"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1028,7 +1161,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6" s="26"/>
     </row>
@@ -1037,7 +1170,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="26"/>
     </row>
@@ -1060,13 +1193,13 @@
         <v>1</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D10" s="23">
         <v>4</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1075,13 +1208,13 @@
         <v>2</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D11" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -1090,13 +1223,13 @@
         <v>3</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -1105,13 +1238,13 @@
         <v>4</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
@@ -1120,13 +1253,13 @@
         <v>5</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D14" s="23">
         <v>7</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1135,13 +1268,13 @@
         <v>6</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D15" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1150,13 +1283,13 @@
         <v>7</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
@@ -1246,7 +1379,7 @@
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1264,7 +1397,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1292,12 +1425,12 @@
       <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1311,7 +1444,7 @@
         <v>20</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J3" s="17">
         <v>235</v>
@@ -1321,15 +1454,15 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="35"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J4" s="3">
         <v>235</v>
@@ -1339,10 +1472,10 @@
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="37"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1355,7 +1488,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E6" s="26"/>
     </row>
@@ -1364,7 +1497,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="26"/>
     </row>
@@ -1387,11 +1520,11 @@
         <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1400,11 +1533,11 @@
         <v>2</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1413,11 +1546,11 @@
         <v>3</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1426,11 +1559,11 @@
         <v>4</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1439,11 +1572,11 @@
         <v>5</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1452,11 +1585,11 @@
         <v>6</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1465,11 +1598,11 @@
         <v>7</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1478,11 +1611,11 @@
         <v>8</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1491,11 +1624,11 @@
         <v>9</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1504,11 +1637,11 @@
         <v>10</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1517,11 +1650,11 @@
         <v>11</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
@@ -1602,7 +1735,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1631,12 +1764,12 @@
       <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1650,7 +1783,7 @@
         <v>20</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J3" s="17">
         <v>235</v>
@@ -1660,15 +1793,15 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="35"/>
+      <c r="E4" s="28"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J4" s="3">
         <v>235</v>
@@ -1678,10 +1811,10 @@
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="D5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="37"/>
+      <c r="E5" s="31"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1694,7 +1827,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6" s="26"/>
     </row>
@@ -1703,7 +1836,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="26"/>
     </row>
@@ -1726,13 +1859,13 @@
         <v>1</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
@@ -1741,13 +1874,13 @@
         <v>2</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -1756,13 +1889,13 @@
         <v>3</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1771,13 +1904,13 @@
         <v>4</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1786,13 +1919,13 @@
         <v>5</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1801,13 +1934,13 @@
         <v>6</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1816,13 +1949,13 @@
         <v>7</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1831,13 +1964,13 @@
         <v>8</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1846,13 +1979,13 @@
         <v>9</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1861,13 +1994,13 @@
         <v>10</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1876,13 +2009,13 @@
         <v>11</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1891,13 +2024,13 @@
         <v>12</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
@@ -2005,7 +2138,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
@@ -2014,10 +2147,9 @@
   <cols>
     <col min="1" max="1" width="8.88671875" style="6"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.88671875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" style="6" customWidth="1"/>
+    <col min="4" max="5" width="23.88671875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="22.77734375" style="6" customWidth="1"/>
     <col min="7" max="8" width="8.88671875" style="6"/>
     <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="6"/>
@@ -2035,12 +2167,12 @@
       <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -2053,26 +2185,38 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
+      <c r="I3" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="17">
+        <v>235</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
+      <c r="D4" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="28"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="40" t="s">
+        <v>111</v>
+      </c>
+      <c r="J4" s="3">
+        <v>235</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="26"/>
+      <c r="D5" s="26" t="s">
+        <v>108</v>
+      </c>
       <c r="E5" s="26"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
@@ -2085,7 +2229,9 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="26"/>
+      <c r="D6" s="26" t="s">
+        <v>109</v>
+      </c>
       <c r="E6" s="26"/>
       <c r="F6" s="20"/>
     </row>
@@ -2106,94 +2252,166 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C17" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="72" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="C18" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
@@ -2317,7 +2535,7 @@
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="C32" s="38" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="D32" s="39"/>
       <c r="E32" s="39"/>

</xml_diff>